<commit_message>
Refactor About section: modern compact layout with structured tech stack and full-width Mermaid diagram
</commit_message>
<xml_diff>
--- a/reports/downloads/bbm_diffusion.xlsx
+++ b/reports/downloads/bbm_diffusion.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8784"/>
+  <dimension ref="A1:B8796"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -70708,6 +70708,102 @@
         <v>28</v>
       </c>
     </row>
+    <row r="8785">
+      <c r="A8785" s="2" t="n">
+        <v>46040</v>
+      </c>
+      <c r="B8785" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8786">
+      <c r="A8786" s="2" t="n">
+        <v>46041</v>
+      </c>
+      <c r="B8786" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8787">
+      <c r="A8787" s="2" t="n">
+        <v>46042</v>
+      </c>
+      <c r="B8787" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8788">
+      <c r="A8788" s="2" t="n">
+        <v>46043</v>
+      </c>
+      <c r="B8788" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8789">
+      <c r="A8789" s="2" t="n">
+        <v>46044</v>
+      </c>
+      <c r="B8789" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8790">
+      <c r="A8790" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="B8790" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8791">
+      <c r="A8791" s="2" t="n">
+        <v>46046</v>
+      </c>
+      <c r="B8791" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8792">
+      <c r="A8792" s="2" t="n">
+        <v>46047</v>
+      </c>
+      <c r="B8792" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8793">
+      <c r="A8793" s="2" t="n">
+        <v>46048</v>
+      </c>
+      <c r="B8793" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8794">
+      <c r="A8794" s="2" t="n">
+        <v>46049</v>
+      </c>
+      <c r="B8794" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8795">
+      <c r="A8795" s="2" t="n">
+        <v>46050</v>
+      </c>
+      <c r="B8795" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8796">
+      <c r="A8796" s="2" t="n">
+        <v>46051</v>
+      </c>
+      <c r="B8796" t="n">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update dashboard with latest data and AI analysis
</commit_message>
<xml_diff>
--- a/reports/downloads/bbm_diffusion.xlsx
+++ b/reports/downloads/bbm_diffusion.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Fix OSII ETL to extract all banks per country, add OSII AI analysis, update About section, fix Mermaid diagram
</commit_message>
<xml_diff>
--- a/reports/downloads/bbm_diffusion.xlsx
+++ b/reports/downloads/bbm_diffusion.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8801"/>
+  <dimension ref="A1:B8802"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -70844,6 +70844,14 @@
         <v>28</v>
       </c>
     </row>
+    <row r="8802">
+      <c r="A8802" s="2" t="n">
+        <v>46057</v>
+      </c>
+      <c r="B8802" t="n">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update: OSII table improvements, Capital Buffer Stack x-axis fix, Mermaid diagram fix, Navigation improvements, BBM section reorganization
</commit_message>
<xml_diff>
--- a/reports/downloads/bbm_diffusion.xlsx
+++ b/reports/downloads/bbm_diffusion.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8802"/>
+  <dimension ref="A1:B8808"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -70852,6 +70852,54 @@
         <v>28</v>
       </c>
     </row>
+    <row r="8803">
+      <c r="A8803" s="2" t="n">
+        <v>46058</v>
+      </c>
+      <c r="B8803" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8804">
+      <c r="A8804" s="2" t="n">
+        <v>46059</v>
+      </c>
+      <c r="B8804" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8805">
+      <c r="A8805" s="2" t="n">
+        <v>46060</v>
+      </c>
+      <c r="B8805" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8806">
+      <c r="A8806" s="2" t="n">
+        <v>46061</v>
+      </c>
+      <c r="B8806" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8807">
+      <c r="A8807" s="2" t="n">
+        <v>46062</v>
+      </c>
+      <c r="B8807" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8808">
+      <c r="A8808" s="2" t="n">
+        <v>46063</v>
+      </c>
+      <c r="B8808" t="n">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
refactor: Move bbm.py and utils.py functions to package modules
- Move bbm.py functions to bbm/ package:
  - build_bbm_matrix_html -> bbm/matrix_builder.py
  - build_dti_lti_items -> bbm/dti_lti/items_builder.py
  - build_dti_lti_eu_list_html -> bbm/dti_lti/list_builder.py
  - extract_ltv_details_regex -> bbm/ltv_legacy.py (compatibility)

- Move utils.py functions to utils/ package:
  - SuppressOutput -> utils/output.py
  - ensure_dirs -> utils/paths.py
  - download_file_safely -> utils/download.py
  - clean_columns, find_header_row, extract_rate -> utils/dataframe.py
  - create_download_link -> utils/html.py

- Update all imports:
  - pipeline/stages/bbm_stage.py
  - scripts/test_*.py
  - bbm/dti_lti_builder.py

- Keep bbm.py and utils.py as deprecated compatibility wrappers

Benefits:
- Eliminates circular import issues
- Better code organization
- Easier maintenance
- Backward compatibility preserved
</commit_message>
<xml_diff>
--- a/reports/downloads/bbm_diffusion.xlsx
+++ b/reports/downloads/bbm_diffusion.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8808"/>
+  <dimension ref="A1:B8809"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -70900,6 +70900,14 @@
         <v>28</v>
       </c>
     </row>
+    <row r="8809">
+      <c r="A8809" s="2" t="n">
+        <v>46064</v>
+      </c>
+      <c r="B8809" t="n">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: Redesign Country Profile page with modern UI
- Add 4 top key measure cards (CCyB, SyRB, O-SII, BBM) with icons and status badges
- Add period selector (1Y, 5Y, Max) to Historical Evolution chart
- Add AI Key Inflection Points timeline card
- Convert Active Measures to tabbed interface (Borrower-Based, Capital-Based, Liquidity)
- Display BBM measures as individual cards with icons and status badges
- Update CSS with new modern design styles
- Fix Mermaid diagram syntax for version 10.9.5
- Filter active measures to show only active/effective tools
- Group measures by type (one card per type with all active measures inside)
</commit_message>
<xml_diff>
--- a/reports/downloads/bbm_diffusion.xlsx
+++ b/reports/downloads/bbm_diffusion.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8809"/>
+  <dimension ref="A1:B8810"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -70908,6 +70908,14 @@
         <v>28</v>
       </c>
     </row>
+    <row r="8810">
+      <c r="A8810" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="B8810" t="n">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Supabase database to Mermaid diagram and update Country Profiles display
</commit_message>
<xml_diff>
--- a/reports/downloads/bbm_diffusion.xlsx
+++ b/reports/downloads/bbm_diffusion.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8810"/>
+  <dimension ref="A1:B8811"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -70916,6 +70916,14 @@
         <v>28</v>
       </c>
     </row>
+    <row r="8811">
+      <c r="A8811" s="2" t="n">
+        <v>46066</v>
+      </c>
+      <c r="B8811" t="n">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Capital stack: ISO2 x-axis, max O-SII/G-SII scale; CCyB historical change-only + step; country profile step charts; migrations 013/014; cache in .gitignore
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/reports/downloads/bbm_diffusion.xlsx
+++ b/reports/downloads/bbm_diffusion.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8811"/>
+  <dimension ref="A1:B8815"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -70924,6 +70924,38 @@
         <v>28</v>
       </c>
     </row>
+    <row r="8812">
+      <c r="A8812" s="2" t="n">
+        <v>46067</v>
+      </c>
+      <c r="B8812" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8813">
+      <c r="A8813" s="2" t="n">
+        <v>46068</v>
+      </c>
+      <c r="B8813" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8814">
+      <c r="A8814" s="2" t="n">
+        <v>46069</v>
+      </c>
+      <c r="B8814" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8815">
+      <c r="A8815" s="2" t="n">
+        <v>46070</v>
+      </c>
+      <c r="B8815" t="n">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Publish pipeline: country profile flags, CCyB/SyRB/visual fixes, improvement suggestions doc
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/reports/downloads/bbm_diffusion.xlsx
+++ b/reports/downloads/bbm_diffusion.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8815"/>
+  <dimension ref="A1:B8816"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -70956,6 +70956,14 @@
         <v>28</v>
       </c>
     </row>
+    <row r="8816">
+      <c r="A8816" s="2" t="n">
+        <v>46071</v>
+      </c>
+      <c r="B8816" t="n">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>